<commit_message>
MAX PROFIT MODE: Andrew Aziz strategy + aggressive config, new features
</commit_message>
<xml_diff>
--- a/trade_history.xlsx
+++ b/trade_history.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3392,6 +3392,3249 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>12:19:00</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>531.11</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>525.8099999999999</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>157</v>
+      </c>
+      <c r="I62" s="4" t="n">
+        <v>-832.1</v>
+      </c>
+      <c r="J62" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>12:54:00</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>212.22</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>213.33</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>393</v>
+      </c>
+      <c r="I63" s="8" t="n">
+        <v>436.23</v>
+      </c>
+      <c r="J63" s="3" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>13:41:00</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>161.65</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>162.67</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>516</v>
+      </c>
+      <c r="I64" s="8" t="n">
+        <v>526.3200000000001</v>
+      </c>
+      <c r="J64" s="3" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>13:49:00</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>714.42</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>715.15</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="I65" s="8" t="n">
+        <v>84.68000000000001</v>
+      </c>
+      <c r="J65" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>13:57:00</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>SCHW</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>90.45999999999999</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>923</v>
+      </c>
+      <c r="I66" s="4" t="n">
+        <v>-239.98</v>
+      </c>
+      <c r="J66" s="3" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>14:02:00</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>213.43</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>214.7</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>391</v>
+      </c>
+      <c r="I67" s="8" t="n">
+        <v>496.57</v>
+      </c>
+      <c r="J67" s="3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>14:19:00</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>424.82</v>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>425.98</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>196</v>
+      </c>
+      <c r="I68" s="8" t="n">
+        <v>227.36</v>
+      </c>
+      <c r="J68" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>14:24:00</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>25.45</v>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>25.57</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>3282</v>
+      </c>
+      <c r="I69" s="8" t="n">
+        <v>393.84</v>
+      </c>
+      <c r="J69" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>14:24:00</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>162.54</v>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>161.59</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>514</v>
+      </c>
+      <c r="I70" s="4" t="n">
+        <v>-488.3</v>
+      </c>
+      <c r="J70" s="3" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>14:49:00</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>215.04</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>216.33</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>388</v>
+      </c>
+      <c r="I71" s="8" t="n">
+        <v>500.52</v>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>14:49:00</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>25.57</v>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>25.46</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>3267</v>
+      </c>
+      <c r="I72" s="4" t="n">
+        <v>-359.37</v>
+      </c>
+      <c r="J72" s="3" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>SCHW</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>90.72</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>90.55</v>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>920</v>
+      </c>
+      <c r="I73" s="4" t="n">
+        <v>-156.4</v>
+      </c>
+      <c r="J73" s="3" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>15:01:00</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>664.0700000000001</v>
+      </c>
+      <c r="G74" s="3" t="n">
+        <v>663.21</v>
+      </c>
+      <c r="H74" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="I74" s="4" t="n">
+        <v>-107.5</v>
+      </c>
+      <c r="J74" s="3" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>15:01:00</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>62.58</v>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>62.35</v>
+      </c>
+      <c r="H75" s="3" t="n">
+        <v>1335</v>
+      </c>
+      <c r="I75" s="4" t="n">
+        <v>-307.05</v>
+      </c>
+      <c r="J75" s="3" t="n">
+        <v>-0.37</v>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>15:09:00</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>310.82</v>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>311.42</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="I76" s="8" t="n">
+        <v>160.8</v>
+      </c>
+      <c r="J76" s="3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>15:17:00</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>14.41</v>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>14.78</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>5798</v>
+      </c>
+      <c r="I77" s="8" t="n">
+        <v>2145.26</v>
+      </c>
+      <c r="J77" s="3" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>15:18:00</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>426.25</v>
+      </c>
+      <c r="G78" s="3" t="n">
+        <v>425.19</v>
+      </c>
+      <c r="H78" s="3" t="n">
+        <v>196</v>
+      </c>
+      <c r="I78" s="4" t="n">
+        <v>-207.76</v>
+      </c>
+      <c r="J78" s="3" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>15:24:00</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>MRNA</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>POWER_HOUR</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>48.63</v>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>48.8</v>
+      </c>
+      <c r="H79" s="3" t="n">
+        <v>1718</v>
+      </c>
+      <c r="I79" s="4" t="n">
+        <v>-292.06</v>
+      </c>
+      <c r="J79" s="3" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>15:29:00</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>OMER</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>POWER_HOUR</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>14.765</v>
+      </c>
+      <c r="G80" s="3" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="H80" s="3" t="n">
+        <v>5658</v>
+      </c>
+      <c r="I80" s="8" t="n">
+        <v>480.93</v>
+      </c>
+      <c r="J80" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>15:41:00</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>25.46</v>
+      </c>
+      <c r="G81" s="3" t="n">
+        <v>25.61</v>
+      </c>
+      <c r="H81" s="3" t="n">
+        <v>3281</v>
+      </c>
+      <c r="I81" s="8" t="n">
+        <v>492.15</v>
+      </c>
+      <c r="J81" s="3" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>15:43:00</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>UVXY</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>POWER_HOUR</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>38.16</v>
+      </c>
+      <c r="G82" s="3" t="n">
+        <v>37.94</v>
+      </c>
+      <c r="H82" s="3" t="n">
+        <v>2189</v>
+      </c>
+      <c r="I82" s="8" t="n">
+        <v>481.58</v>
+      </c>
+      <c r="J82" s="3" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>12:41:00</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>366.69</v>
+      </c>
+      <c r="G83" s="3" t="n">
+        <v>368.95</v>
+      </c>
+      <c r="H83" s="3" t="n">
+        <v>237</v>
+      </c>
+      <c r="I83" s="8" t="n">
+        <v>535.62</v>
+      </c>
+      <c r="J83" s="3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>13:16:00</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>SQQQ</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>54.72</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>54.49</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>1592</v>
+      </c>
+      <c r="I84" s="4" t="n">
+        <v>-366.16</v>
+      </c>
+      <c r="J84" s="3" t="n">
+        <v>-0.42</v>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>13:43:00</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>58.89</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>58.72</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>1479</v>
+      </c>
+      <c r="I85" s="4" t="n">
+        <v>-251.43</v>
+      </c>
+      <c r="J85" s="3" t="n">
+        <v>-0.29</v>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>13:45:00</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>NIO</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>6.27</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>13894</v>
+      </c>
+      <c r="I86" s="8" t="n">
+        <v>694.7</v>
+      </c>
+      <c r="J86" s="3" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>13:51:00</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>189.17</v>
+      </c>
+      <c r="G87" s="3" t="n">
+        <v>188.83</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="I87" s="4" t="n">
+        <v>-156.4</v>
+      </c>
+      <c r="J87" s="3" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>14:23:00</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>MSFT</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>428.4</v>
+      </c>
+      <c r="G88" s="3" t="n">
+        <v>426.93</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>203</v>
+      </c>
+      <c r="I88" s="4" t="n">
+        <v>-298.41</v>
+      </c>
+      <c r="J88" s="3" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>15:36:00</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>POWER_HOUR</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>195.14</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>194.54</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>446</v>
+      </c>
+      <c r="I89" s="4" t="n">
+        <v>-267.6</v>
+      </c>
+      <c r="J89" s="3" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>12:10:00</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>61.4</v>
+      </c>
+      <c r="G90" s="3" t="n">
+        <v>61.09</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>1389</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>-430.59</v>
+      </c>
+      <c r="J90" s="3" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="K90" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>12:10:00</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>UVXY</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>37.63</v>
+      </c>
+      <c r="G91" s="3" t="n">
+        <v>38.09</v>
+      </c>
+      <c r="H91" s="3" t="n">
+        <v>2267</v>
+      </c>
+      <c r="I91" s="8" t="n">
+        <v>1042.82</v>
+      </c>
+      <c r="J91" s="3" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>12:12:00</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>SCHW</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="n">
+        <v>90.84</v>
+      </c>
+      <c r="G92" s="3" t="n">
+        <v>90.56999999999999</v>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>939</v>
+      </c>
+      <c r="I92" s="4" t="n">
+        <v>-253.53</v>
+      </c>
+      <c r="J92" s="3" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>12:13:00</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>659.89</v>
+      </c>
+      <c r="G93" s="3" t="n">
+        <v>658.77</v>
+      </c>
+      <c r="H93" s="3" t="n">
+        <v>129</v>
+      </c>
+      <c r="I93" s="4" t="n">
+        <v>-144.48</v>
+      </c>
+      <c r="J93" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>15:03:00</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>UVXY</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>POWER_HOUR</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="G94" s="3" t="n">
+        <v>38.37</v>
+      </c>
+      <c r="H94" s="3" t="n">
+        <v>2216</v>
+      </c>
+      <c r="I94" s="4" t="n">
+        <v>-288.08</v>
+      </c>
+      <c r="J94" s="3" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>15:24:00</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>SOFI</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>POWER_HOUR</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="G95" s="3" t="n">
+        <v>15.68</v>
+      </c>
+      <c r="H95" s="3" t="n">
+        <v>5465</v>
+      </c>
+      <c r="I95" s="4" t="n">
+        <v>-382.55</v>
+      </c>
+      <c r="J95" s="3" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="K95" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>09:46:00</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>711.58</v>
+      </c>
+      <c r="G96" s="3" t="n">
+        <v>713.66</v>
+      </c>
+      <c r="H96" s="3" t="n">
+        <v>117</v>
+      </c>
+      <c r="I96" s="8" t="n">
+        <v>243.36</v>
+      </c>
+      <c r="J96" s="3" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>11:47:00</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>PDD</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="G97" s="3" t="n">
+        <v>99.16</v>
+      </c>
+      <c r="H97" s="3" t="n">
+        <v>843</v>
+      </c>
+      <c r="I97" s="4" t="n">
+        <v>-286.62</v>
+      </c>
+      <c r="J97" s="3" t="n">
+        <v>-0.34</v>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>12:52:00</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>24.69</v>
+      </c>
+      <c r="G98" s="3" t="n">
+        <v>24.59</v>
+      </c>
+      <c r="H98" s="3" t="n">
+        <v>3363</v>
+      </c>
+      <c r="I98" s="4" t="n">
+        <v>-336.3</v>
+      </c>
+      <c r="J98" s="3" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>13:01:00</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>BX</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="n">
+        <v>125.71</v>
+      </c>
+      <c r="G99" s="3" t="n">
+        <v>125.07</v>
+      </c>
+      <c r="H99" s="3" t="n">
+        <v>660</v>
+      </c>
+      <c r="I99" s="4" t="n">
+        <v>-422.4</v>
+      </c>
+      <c r="J99" s="3" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="K99" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>13:06:00</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="n">
+        <v>273.43</v>
+      </c>
+      <c r="G100" s="3" t="n">
+        <v>272.46</v>
+      </c>
+      <c r="H100" s="3" t="n">
+        <v>303</v>
+      </c>
+      <c r="I100" s="4" t="n">
+        <v>-293.91</v>
+      </c>
+      <c r="J100" s="3" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>13:07:00</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>DIA</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>495.85</v>
+      </c>
+      <c r="G101" s="3" t="n">
+        <v>495.22</v>
+      </c>
+      <c r="H101" s="3" t="n">
+        <v>167</v>
+      </c>
+      <c r="I101" s="4" t="n">
+        <v>-105.21</v>
+      </c>
+      <c r="J101" s="3" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>13:14:00</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>UNH</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="n">
+        <v>370.48</v>
+      </c>
+      <c r="G102" s="3" t="n">
+        <v>371.78</v>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>224</v>
+      </c>
+      <c r="I102" s="8" t="n">
+        <v>291.2</v>
+      </c>
+      <c r="J102" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>13:17:00</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>XOM</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>155.3</v>
+      </c>
+      <c r="G103" s="3" t="n">
+        <v>154.93</v>
+      </c>
+      <c r="H103" s="3" t="n">
+        <v>534</v>
+      </c>
+      <c r="I103" s="4" t="n">
+        <v>-197.58</v>
+      </c>
+      <c r="J103" s="3" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>13:19:00</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>DIS</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>102.86</v>
+      </c>
+      <c r="G104" s="3" t="n">
+        <v>102.68</v>
+      </c>
+      <c r="H104" s="3" t="n">
+        <v>807</v>
+      </c>
+      <c r="I104" s="4" t="n">
+        <v>-145.26</v>
+      </c>
+      <c r="J104" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>13:36:00</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>LCID</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="G105" s="3" t="n">
+        <v>6.115</v>
+      </c>
+      <c r="H105" s="3" t="n">
+        <v>13459</v>
+      </c>
+      <c r="I105" s="4" t="n">
+        <v>-740.24</v>
+      </c>
+      <c r="J105" s="3" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>12:36:00</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="n">
+        <v>53.59</v>
+      </c>
+      <c r="G106" s="3" t="n">
+        <v>53.53</v>
+      </c>
+      <c r="H106" s="3" t="n">
+        <v>1531</v>
+      </c>
+      <c r="I106" s="4" t="n">
+        <v>-91.86</v>
+      </c>
+      <c r="J106" s="3" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="K106" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>12:39:00</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>53.51</v>
+      </c>
+      <c r="G107" s="3" t="n">
+        <v>53.44</v>
+      </c>
+      <c r="H107" s="3" t="n">
+        <v>1534</v>
+      </c>
+      <c r="I107" s="4" t="n">
+        <v>-107.38</v>
+      </c>
+      <c r="J107" s="3" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="K107" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>12:41:00</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>MRVL</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>165.95</v>
+      </c>
+      <c r="G108" s="3" t="n">
+        <v>164.99</v>
+      </c>
+      <c r="H108" s="3" t="n">
+        <v>494</v>
+      </c>
+      <c r="I108" s="4" t="n">
+        <v>-474.24</v>
+      </c>
+      <c r="J108" s="3" t="n">
+        <v>-0.58</v>
+      </c>
+      <c r="K108" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>12:41:00</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>VWAP_RECLAIM</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>58.97</v>
+      </c>
+      <c r="G109" s="3" t="n">
+        <v>59.16</v>
+      </c>
+      <c r="H109" s="3" t="n">
+        <v>1392</v>
+      </c>
+      <c r="I109" s="8" t="n">
+        <v>264.48</v>
+      </c>
+      <c r="J109" s="3" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>12:45:00</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>313.06</v>
+      </c>
+      <c r="G110" s="3" t="n">
+        <v>312.54</v>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>262</v>
+      </c>
+      <c r="I110" s="4" t="n">
+        <v>-136.24</v>
+      </c>
+      <c r="J110" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="K110" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>12:47:00</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>93.41</v>
+      </c>
+      <c r="G111" s="3" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="H111" s="3" t="n">
+        <v>878</v>
+      </c>
+      <c r="I111" s="4" t="n">
+        <v>-184.38</v>
+      </c>
+      <c r="J111" s="3" t="n">
+        <v>-0.22</v>
+      </c>
+      <c r="K111" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>13:06:00</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="n">
+        <v>25.19</v>
+      </c>
+      <c r="G112" s="3" t="n">
+        <v>25.35</v>
+      </c>
+      <c r="H112" s="3" t="n">
+        <v>3258</v>
+      </c>
+      <c r="I112" s="8" t="n">
+        <v>521.28</v>
+      </c>
+      <c r="J112" s="3" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="K112" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>13:07:00</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>UVXY</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="n">
+        <v>36.44</v>
+      </c>
+      <c r="G113" s="3" t="n">
+        <v>36.19</v>
+      </c>
+      <c r="H113" s="3" t="n">
+        <v>2252</v>
+      </c>
+      <c r="I113" s="4" t="n">
+        <v>-563</v>
+      </c>
+      <c r="J113" s="3" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>13:21:00</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="n">
+        <v>25.41</v>
+      </c>
+      <c r="G114" s="3" t="n">
+        <v>25.62</v>
+      </c>
+      <c r="H114" s="3" t="n">
+        <v>8090</v>
+      </c>
+      <c r="I114" s="8" t="n">
+        <v>1698.9</v>
+      </c>
+      <c r="J114" s="3" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="K114" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>14:01:00</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="n">
+        <v>421.95</v>
+      </c>
+      <c r="G115" s="3" t="n">
+        <v>422.91</v>
+      </c>
+      <c r="H115" s="3" t="n">
+        <v>488</v>
+      </c>
+      <c r="I115" s="8" t="n">
+        <v>468.48</v>
+      </c>
+      <c r="J115" s="3" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="K115" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>14:03:00</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="n">
+        <v>613.83</v>
+      </c>
+      <c r="G116" s="3" t="n">
+        <v>612.1</v>
+      </c>
+      <c r="H116" s="3" t="n">
+        <v>335</v>
+      </c>
+      <c r="I116" s="4" t="n">
+        <v>-579.55</v>
+      </c>
+      <c r="J116" s="3" t="n">
+        <v>-0.28</v>
+      </c>
+      <c r="K116" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>14:17:00</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="n">
+        <v>425.2</v>
+      </c>
+      <c r="G117" s="3" t="n">
+        <v>424.75</v>
+      </c>
+      <c r="H117" s="3" t="n">
+        <v>483</v>
+      </c>
+      <c r="I117" s="4" t="n">
+        <v>-217.35</v>
+      </c>
+      <c r="J117" s="3" t="n">
+        <v>-0.11</v>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>14:22:00</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="G118" s="3" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="H118" s="3" t="n">
+        <v>7476</v>
+      </c>
+      <c r="I118" s="4" t="n">
+        <v>-747.6</v>
+      </c>
+      <c r="J118" s="3" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>14:27:00</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>UVXY</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="n">
+        <v>36.46</v>
+      </c>
+      <c r="G119" s="3" t="n">
+        <v>36.62</v>
+      </c>
+      <c r="H119" s="3" t="n">
+        <v>5638</v>
+      </c>
+      <c r="I119" s="8" t="n">
+        <v>902.08</v>
+      </c>
+      <c r="J119" s="3" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>14:29:00</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>TQQQ</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="n">
+        <v>65.65000000000001</v>
+      </c>
+      <c r="G120" s="3" t="n">
+        <v>65.48999999999999</v>
+      </c>
+      <c r="H120" s="3" t="n">
+        <v>3131</v>
+      </c>
+      <c r="I120" s="4" t="n">
+        <v>-500.96</v>
+      </c>
+      <c r="J120" s="3" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="K120" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>14:42:00</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="n">
+        <v>362.16</v>
+      </c>
+      <c r="G121" s="3" t="n">
+        <v>360.74</v>
+      </c>
+      <c r="H121" s="3" t="n">
+        <v>567</v>
+      </c>
+      <c r="I121" s="4" t="n">
+        <v>-805.14</v>
+      </c>
+      <c r="J121" s="3" t="n">
+        <v>-0.39</v>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>14:51:00</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="n">
+        <v>384.9</v>
+      </c>
+      <c r="G122" s="3" t="n">
+        <v>384.09</v>
+      </c>
+      <c r="H122" s="3" t="n">
+        <v>534</v>
+      </c>
+      <c r="I122" s="4" t="n">
+        <v>-432.54</v>
+      </c>
+      <c r="J122" s="3" t="n">
+        <v>-0.21</v>
+      </c>
+      <c r="K122" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>14:51:00</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>NKE</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="n">
+        <v>44.31</v>
+      </c>
+      <c r="G123" s="3" t="n">
+        <v>44.25</v>
+      </c>
+      <c r="H123" s="3" t="n">
+        <v>4639</v>
+      </c>
+      <c r="I123" s="4" t="n">
+        <v>-278.34</v>
+      </c>
+      <c r="J123" s="3" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>14:58:00</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="n">
+        <v>422.41</v>
+      </c>
+      <c r="G124" s="3" t="n">
+        <v>421.65</v>
+      </c>
+      <c r="H124" s="3" t="n">
+        <v>486</v>
+      </c>
+      <c r="I124" s="4" t="n">
+        <v>-369.36</v>
+      </c>
+      <c r="J124" s="3" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="K124" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>15:01:00</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>GME</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="G125" s="3" t="n">
+        <v>26.68</v>
+      </c>
+      <c r="H125" s="3" t="n">
+        <v>7817</v>
+      </c>
+      <c r="I125" s="8" t="n">
+        <v>2970.46</v>
+      </c>
+      <c r="J125" s="3" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="K125" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>15:03:00</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>SQQQ</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="n">
+        <v>50.22</v>
+      </c>
+      <c r="G126" s="3" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="H126" s="3" t="n">
+        <v>4093</v>
+      </c>
+      <c r="I126" s="8" t="n">
+        <v>695.8099999999999</v>
+      </c>
+      <c r="J126" s="3" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="K126" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>15:07:00</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>AMC</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="n">
+        <v>1.4531</v>
+      </c>
+      <c r="G127" s="3" t="n">
+        <v>1.4865</v>
+      </c>
+      <c r="H127" s="3" t="n">
+        <v>141484</v>
+      </c>
+      <c r="I127" s="8" t="n">
+        <v>4725.57</v>
+      </c>
+      <c r="J127" s="3" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="K127" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>15:26:00</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>OXY</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="n">
+        <v>58.89</v>
+      </c>
+      <c r="G128" s="3" t="n">
+        <v>59.05</v>
+      </c>
+      <c r="H128" s="3" t="n">
+        <v>3491</v>
+      </c>
+      <c r="I128" s="8" t="n">
+        <v>558.5599999999999</v>
+      </c>
+      <c r="J128" s="3" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="K128" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>15:32:00</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="n">
+        <v>99.18000000000001</v>
+      </c>
+      <c r="G129" s="3" t="n">
+        <v>99.65000000000001</v>
+      </c>
+      <c r="H129" s="3" t="n">
+        <v>2072</v>
+      </c>
+      <c r="I129" s="8" t="n">
+        <v>973.84</v>
+      </c>
+      <c r="J129" s="3" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>15:35:00</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>JPM</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="n">
+        <v>313.74</v>
+      </c>
+      <c r="G130" s="3" t="n">
+        <v>314.18</v>
+      </c>
+      <c r="H130" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="I130" s="8" t="n">
+        <v>288.2</v>
+      </c>
+      <c r="J130" s="3" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="K130" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3403,7 +6646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3420,7 +6663,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>60</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4">
@@ -3430,7 +6673,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -3440,7 +6683,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6">
@@ -3451,7 +6694,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>45.0%</t>
+          <t>42.6%</t>
         </is>
       </c>
     </row>
@@ -3462,7 +6705,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>2476.78</v>
+        <v>11933.17</v>
       </c>
     </row>
     <row r="9">
@@ -3512,15 +6755,15 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>45%</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4972.87</v>
+        <v>7945.37</v>
       </c>
     </row>
     <row r="12">
@@ -3548,7 +6791,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -3556,7 +6799,61 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-30</v>
+        <v>-297.78</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>6</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>-1545.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>VWAP_RECLAIM</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>264.48</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>MA_TREND</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>8032.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Retrain model with MTM loss data: blacklist 9 serial losers, inject 84 loss lessons, wire blacklist gate into check_entry
</commit_message>
<xml_diff>
--- a/trade_history.xlsx
+++ b/trade_history.xlsx
@@ -499,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K130"/>
+  <dimension ref="A1:K136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6635,6 +6635,288 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>09:47:00</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>RDDT</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>GAP_FILL</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="n">
+        <v>169.73</v>
+      </c>
+      <c r="G131" s="3" t="n">
+        <v>170.96</v>
+      </c>
+      <c r="H131" s="3" t="n">
+        <v>1181</v>
+      </c>
+      <c r="I131" s="4" t="n">
+        <v>-1452.63</v>
+      </c>
+      <c r="J131" s="3" t="n">
+        <v>-0.72</v>
+      </c>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>09:50:00</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>LLY</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>GAP_FILL</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="n">
+        <v>957.54</v>
+      </c>
+      <c r="G132" s="3" t="n">
+        <v>967.35</v>
+      </c>
+      <c r="H132" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="I132" s="4" t="n">
+        <v>-2050.29</v>
+      </c>
+      <c r="J132" s="3" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="K132" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>09:54:00</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>INTC</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>GAP_FILL</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="n">
+        <v>98.54000000000001</v>
+      </c>
+      <c r="G133" s="3" t="n">
+        <v>96.73</v>
+      </c>
+      <c r="H133" s="3" t="n">
+        <v>2035</v>
+      </c>
+      <c r="I133" s="8" t="n">
+        <v>3683.35</v>
+      </c>
+      <c r="J133" s="3" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>10:03:00</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>COIN</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>GAP_FILL</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="n">
+        <v>199.25</v>
+      </c>
+      <c r="G134" s="3" t="n">
+        <v>200.97</v>
+      </c>
+      <c r="H134" s="3" t="n">
+        <v>1006</v>
+      </c>
+      <c r="I134" s="4" t="n">
+        <v>-1730.32</v>
+      </c>
+      <c r="J134" s="3" t="n">
+        <v>-0.86</v>
+      </c>
+      <c r="K134" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>11:35:00</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>UVXY</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>RSI_EXTREME</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="n">
+        <v>37.02</v>
+      </c>
+      <c r="G135" s="3" t="n">
+        <v>37.42</v>
+      </c>
+      <c r="H135" s="3" t="n">
+        <v>1057</v>
+      </c>
+      <c r="I135" s="4" t="n">
+        <v>-422.8</v>
+      </c>
+      <c r="J135" s="3" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="K135" s="3" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>11:37:00</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>ORB</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="n">
+        <v>417.92</v>
+      </c>
+      <c r="G136" s="3" t="n">
+        <v>414.62</v>
+      </c>
+      <c r="H136" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="I136" s="8" t="n">
+        <v>306.9</v>
+      </c>
+      <c r="J136" s="3" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="K136" s="3" t="inlineStr">
+        <is>
+          <t>TARGET1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6663,7 +6945,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>129</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
@@ -6673,7 +6955,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5">
@@ -6683,7 +6965,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6">
@@ -6694,7 +6976,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>42.6%</t>
+          <t>42.2%</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6987,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>11933.17</v>
+        <v>10267.38</v>
       </c>
     </row>
     <row r="9">
@@ -6755,7 +7037,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -6763,7 +7045,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7945.37</v>
+        <v>8252.27</v>
       </c>
     </row>
     <row r="12">
@@ -6773,15 +7055,15 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-2402.88</v>
+        <v>-3952.77</v>
       </c>
     </row>
     <row r="13">
@@ -6809,7 +7091,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -6817,7 +7099,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-1545.8</v>
+        <v>-1968.6</v>
       </c>
     </row>
     <row r="15">

</xml_diff>